<commit_message>
continue in detailing components
</commit_message>
<xml_diff>
--- a/documents/00. Database-ERD-Schemas.xlsx
+++ b/documents/00. Database-ERD-Schemas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://petrosea-my.sharepoint.com/personal/harry_kurniansyah_petrosea_com/Documents/Documents/2_Harry_Kurniansyah_Docs/0_Very_Personal/MechSense/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="381" documentId="11_F25DC773A252ABDACC104813B1DE57565ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80B5E142-709F-4C5A-9F3A-3CEE52E79138}"/>
+  <xr:revisionPtr revIDLastSave="383" documentId="11_F25DC773A252ABDACC104813B1DE57565ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93A274FC-942C-461E-98DC-7D3C890B8EDB}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table - Site Master" sheetId="2" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="Table - Model Master" sheetId="5" r:id="rId4"/>
     <sheet name="Table - Equipment Master" sheetId="6" r:id="rId5"/>
     <sheet name="Table - Hour Meter History" sheetId="7" r:id="rId6"/>
+    <sheet name="Table - Component Master" sheetId="8" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -1426,4 +1427,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F56EE3AE-FFAB-472A-BB92-6D07A37EC867}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
finalize models and schemas
</commit_message>
<xml_diff>
--- a/documents/00. Database-ERD-Schemas.xlsx
+++ b/documents/00. Database-ERD-Schemas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://petrosea-my.sharepoint.com/personal/harry_kurniansyah_petrosea_com/Documents/Documents/2_Harry_Kurniansyah_Docs/0_Very_Personal/MechSense/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="383" documentId="11_F25DC773A252ABDACC104813B1DE57565ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93A274FC-942C-461E-98DC-7D3C890B8EDB}"/>
+  <xr:revisionPtr revIDLastSave="455" documentId="11_F25DC773A252ABDACC104813B1DE57565ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4149FFF4-3DDC-4D60-8AB6-6994953FC165}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table - Site Master" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,9 @@
     <sheet name="Table - Equipment Master" sheetId="6" r:id="rId5"/>
     <sheet name="Table - Hour Meter History" sheetId="7" r:id="rId6"/>
     <sheet name="Table - Component Master" sheetId="8" r:id="rId7"/>
+    <sheet name="Table - Model Component Master" sheetId="9" r:id="rId8"/>
+    <sheet name="Table - Component Instance" sheetId="10" r:id="rId9"/>
+    <sheet name="Tabel - Equipment Status Log" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="89">
   <si>
     <t>{uuid}</t>
   </si>
@@ -297,6 +300,46 @@
   </si>
   <si>
     <t>API_SYSTEM</t>
+  </si>
+  <si>
+    <t>component_code
+(VARCHAR)</t>
+  </si>
+  <si>
+    <t>DT0123</t>
+  </si>
+  <si>
+    <t>component_name
+(VARCHAR)</t>
+  </si>
+  <si>
+    <t>component_master_id
+(UUID)</t>
+  </si>
+  <si>
+    <t>target_life_hm
+(UUID)</t>
+  </si>
+  <si>
+    <t>master_id</t>
+  </si>
+  <si>
+    <t>equipment_id</t>
+  </si>
+  <si>
+    <t>serial_number</t>
+  </si>
+  <si>
+    <t>installed_date</t>
+  </si>
+  <si>
+    <t>installed_equipment_hm</t>
+  </si>
+  <si>
+    <t>current_component_hm</t>
+  </si>
+  <si>
+    <t>status</t>
   </si>
 </sst>
 </file>
@@ -722,6 +765,15 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{317A0D0E-7732-40F6-A8D3-3A3912AFC7BF}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F10698-B894-4157-9D90-FB68318B125C}">
   <dimension ref="A1:H6"/>
@@ -1325,6 +1377,9 @@
       <c r="D2" t="s">
         <v>69</v>
       </c>
+      <c r="E2" t="s">
+        <v>78</v>
+      </c>
       <c r="F2" s="3">
         <v>45658</v>
       </c>
@@ -1431,9 +1486,167 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F56EE3AE-FFAB-472A-BB92-6D07A37EC867}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
+    <col min="5" max="5" width="9.88671875" customWidth="1"/>
+    <col min="6" max="7" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46162.041666666664</v>
+      </c>
+      <c r="G2" s="1">
+        <v>46162.041666666664</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D67D70-ED5C-422E-987D-DE89222C51A1}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.21875" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F2" s="1">
+        <v>46162.041666666664</v>
+      </c>
+      <c r="G2" s="1">
+        <v>46162.041666666664</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A59117C-1BF4-4906-ABC5-F2C7643F287C}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E1" t="s">
+        <v>85</v>
+      </c>
+      <c r="F1" t="s">
+        <v>86</v>
+      </c>
+      <c r="G1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
develop master data and eqp
</commit_message>
<xml_diff>
--- a/documents/00. Database-ERD-Schemas.xlsx
+++ b/documents/00. Database-ERD-Schemas.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://petrosea-my.sharepoint.com/personal/harry_kurniansyah_petrosea_com/Documents/Documents/2_Harry_Kurniansyah_Docs/0_Very_Personal/MechSense/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="455" documentId="11_F25DC773A252ABDACC104813B1DE57565ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4149FFF4-3DDC-4D60-8AB6-6994953FC165}"/>
+  <xr:revisionPtr revIDLastSave="456" documentId="11_F25DC773A252ABDACC104813B1DE57565ADE58F2" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AE491565-7F9A-4AAE-B649-5A6174320C09}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table - Site Master" sheetId="2" r:id="rId1"/>
@@ -24,10 +24,21 @@
     <sheet name="Table - Component Instance" sheetId="10" r:id="rId9"/>
     <sheet name="Tabel - Equipment Status Log" sheetId="11" r:id="rId10"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -666,6 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2C4114C-3269-42E0-A2EE-B55B0E7032E4}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -767,6 +779,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{317A0D0E-7732-40F6-A8D3-3A3912AFC7BF}">
+  <sheetPr codeName="Sheet10"/>
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
@@ -776,6 +789,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F10698-B894-4157-9D90-FB68318B125C}">
+  <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -935,12 +949,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86B34790-3214-40B1-A3B8-A15FC42E8D0D}">
+  <sheetPr codeName="Sheet3"/>
   <dimension ref="A1:J6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="9.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.109375" customWidth="1"/>
     <col min="7" max="7" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1129,6 +1144,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8729D20B-9EDA-4E99-827A-CDCDA414618E}">
+  <sheetPr codeName="Sheet4"/>
   <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1295,6 +1311,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA848FAC-5F88-4CC3-9D76-3095E418F625}">
+  <sheetPr codeName="Sheet5"/>
   <dimension ref="A1:P2"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1418,6 +1435,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{031EAB8B-E322-4254-9F67-BB8F132B9396}">
+  <sheetPr codeName="Sheet6"/>
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1486,6 +1504,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F56EE3AE-FFAB-472A-BB92-6D07A37EC867}">
+  <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1545,6 +1564,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13D67D70-ED5C-422E-987D-DE89222C51A1}">
+  <sheetPr codeName="Sheet8"/>
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1602,6 +1622,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A59117C-1BF4-4906-ABC5-F2C7643F287C}">
+  <sheetPr codeName="Sheet9"/>
   <dimension ref="A1:H2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>